<commit_message>
Save working baseline before RTS/CTS flow-control optimization
</commit_message>
<xml_diff>
--- a/doc/notes/ro-rl78-maxv-learning.xlsx
+++ b/doc/notes/ro-rl78-maxv-learning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\0_forge\ro-rl78-maxv-learning\doc\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{845FE8D0-A19B-4EF7-AF4D-F3D9E9B2953E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57CC9C05-EBED-40B3-88DE-97FAF23E96F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-225" windowWidth="29040" windowHeight="16440" firstSheet="4" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -32,6 +32,7 @@
     <sheet name="ROM" sheetId="25" r:id="rId17"/>
     <sheet name="FLOW" sheetId="26" r:id="rId18"/>
     <sheet name="DMA" sheetId="27" r:id="rId19"/>
+    <sheet name="BiUART" sheetId="29" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4'!$A$6:$AB$70</definedName>
@@ -8587,6 +8588,1291 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="130" name="テキスト ボックス 129">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BEEBBD13-853F-41AE-8D2E-8A3738D43A45}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4000500" y="3619500"/>
+          <a:ext cx="762000" cy="952500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="19050" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t>USB-UART</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100" baseline="30000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="131" name="直線矢印コネクタ 130">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{121FCA77-CB7E-4BE0-8469-B54DD61CDF6E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="5524500" y="2476500"/>
+          <a:ext cx="0" cy="1524000"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:headEnd type="oval"/>
+          <a:tailEnd type="none"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>184547</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>5953</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="133" name="直線矢印コネクタ 132">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77DBE3D7-EA3F-F320-02C6-70B16D8B9415}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="3042047" y="4191000"/>
+          <a:ext cx="958453" cy="5953"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:headEnd type="triangle"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="134" name="テキスト ボックス 133">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D3C0345-9D52-E837-C1A3-7279387BB5EB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2286000" y="3619500"/>
+          <a:ext cx="762000" cy="952500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="19050" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t>PC</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100" baseline="30000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="136" name="直線矢印コネクタ 135">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DBFCBB62-3922-61EC-E3E6-B715CED46BB8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4762500" y="4000500"/>
+          <a:ext cx="2095500" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:headEnd type="none"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="138" name="テキスト ボックス 137">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{89A400C0-5F2B-CFB9-4518-53D19A02F36F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4572000" y="3810000"/>
+          <a:ext cx="190500" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="800"/>
+            <a:t>TX</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="139" name="直線矢印コネクタ 138">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93D701ED-EB74-4806-FBC0-BAFB91FC1436}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="4762500" y="4381500"/>
+          <a:ext cx="2095500" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:headEnd type="none"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="140" name="テキスト ボックス 139">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34E8E89F-B4D4-67AE-FE3F-256230BA6388}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4572000" y="4191000"/>
+          <a:ext cx="190500" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="800"/>
+            <a:t>RX</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="141" name="テキスト ボックス 140">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{300EB7AF-78BA-3E8F-9CBF-AD3A6EC9F869}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6858000" y="3619500"/>
+          <a:ext cx="762000" cy="952500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="19050" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t>MCU</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100" baseline="30000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="145" name="テキスト ボックス 144">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D3CDDC0-B964-035C-E0DE-FBDE0A538346}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6858000" y="3810000"/>
+          <a:ext cx="190500" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="800"/>
+            <a:t>RX</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="146" name="テキスト ボックス 145">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1B1517A-68FB-BE29-F022-B5E054094D43}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6858000" y="4191000"/>
+          <a:ext cx="762000" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="800"/>
+            <a:t>  TX (Open</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="800" baseline="0"/>
+            <a:t> Drain)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="800"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="147" name="テキスト ボックス 146">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71240E68-2482-76A5-FF2A-FA2C8FF8CD3A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6858000" y="2095500"/>
+          <a:ext cx="762000" cy="952500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="19050" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t>CPLD/FPGA</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100" baseline="30000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="148" name="直線矢印コネクタ 147">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC7088DD-C215-D7B3-53DC-32CEED6F4F1A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="7239000" y="3048000"/>
+          <a:ext cx="0" cy="571500"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:headEnd type="triangle"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="151" name="テキスト ボックス 150">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5039324D-660E-ED19-7429-1C4E90AB9FAD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7239000" y="3238500"/>
+          <a:ext cx="381000" cy="190500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP" sz="800"/>
+            <a:t>JTAG</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="800"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="152" name="テキスト ボックス 151">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48084D97-395A-1B3B-56B6-7FDE487CC651}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6858000" y="2286000"/>
+          <a:ext cx="571500" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="800"/>
+            <a:t>  RX</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="en-US" sz="800" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" altLang="ja-JP" sz="800" baseline="0"/>
+            <a:t>(input)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="800"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="153" name="テキスト ボックス 152">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EE80F22-70E2-3491-507C-054739C85B5F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6858000" y="2667000"/>
+          <a:ext cx="762000" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="800"/>
+            <a:t>  TX (output)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="154" name="直線矢印コネクタ 153">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D6B0105-8877-EC20-ECDF-EDD6C5A5F05B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5524500" y="2476500"/>
+          <a:ext cx="1333500" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:headEnd type="none"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="158" name="直線矢印コネクタ 157">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9EC55C19-2C9E-C57D-D3A7-1EA68B2981A8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6096000" y="2857500"/>
+          <a:ext cx="0" cy="1524000"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:headEnd type="none"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>125016</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>65483</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>71438</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>5952</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="132" name="テキスト ボックス 131">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{97D3A0BD-113E-4B7E-93C9-413474E864A3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="5938242" y="3205757"/>
+          <a:ext cx="321469" cy="136922"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="800"/>
+            <a:t>1k</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ja-JP" sz="800"/>
+            <a:t>Ω</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="800"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="161" name="直線矢印コネクタ 160">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19EA6F74-B291-5D0B-D732-D19853C7FF69}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="6096000" y="2857500"/>
+          <a:ext cx="762000" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:headEnd type="none"/>
+          <a:tailEnd type="none"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -33179,6 +34465,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F29E5D87-F4F7-449C-A476-A67CED2034FA}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28A881EA-E0AB-4311-93A9-080EF2A17ED8}">
   <dimension ref="B2:C4"/>

</xml_diff>

<commit_message>
Keep the 32-bit scan length for compatibility and future long SVF scans; 1-byte saves only ~0.23 s.
</commit_message>
<xml_diff>
--- a/doc/notes/ro-rl78-maxv-learning.xlsx
+++ b/doc/notes/ro-rl78-maxv-learning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\0_forge\ro-rl78-maxv-learning\doc\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57CC9C05-EBED-40B3-88DE-97FAF23E96F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3F4314-C066-40AF-A4B1-7FAF77304B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-225" windowWidth="29040" windowHeight="16440" firstSheet="4" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1898" uniqueCount="750">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1901" uniqueCount="754">
   <si>
     <t>Block Diagram</t>
   </si>
@@ -2867,6 +2867,18 @@
       </rPr>
       <t>(DST0)</t>
     </r>
+  </si>
+  <si>
+    <t>TCK Count *1</t>
+  </si>
+  <si>
+    <t>*1</t>
+  </si>
+  <si>
+    <t>Reducing the scan length field to one byte would save at most approximately 0.23 seconds, less than 10% of the total execution time.</t>
+  </si>
+  <si>
+    <t>The 32-bit length field will therefore be retained to preserve protocol compatibility and support longer SVF scan operations in the future.</t>
   </si>
 </sst>
 </file>
@@ -4509,6 +4521,15 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -4527,13 +4548,97 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="38" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="69" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="33" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="65" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="66" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="57" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="53" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="58" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="61" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="5" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="7" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="24" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="63" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="56" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="70" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="71" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="5" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="25" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="67" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4557,94 +4662,10 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="33" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="5" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="16" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="64" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="65" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="66" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="63" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="56" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="70" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="71" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="5" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="57" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="53" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="60" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="59" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="58" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="62" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="61" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="38" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="69" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4658,15 +4679,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -25576,11 +25588,11 @@
       <c r="H4" s="16" t="s">
         <v>371</v>
       </c>
-      <c r="J4" s="165" t="s">
+      <c r="J4" s="168" t="s">
         <v>664</v>
       </c>
-      <c r="K4" s="165"/>
-      <c r="L4" s="165"/>
+      <c r="K4" s="168"/>
+      <c r="L4" s="168"/>
     </row>
     <row r="5" spans="2:12">
       <c r="B5" s="14">
@@ -27956,32 +27968,32 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:20">
-      <c r="B4" s="169"/>
-      <c r="C4" s="169"/>
-      <c r="D4" s="169"/>
-      <c r="E4" s="169" t="s">
+      <c r="B4" s="172"/>
+      <c r="C4" s="172"/>
+      <c r="D4" s="172"/>
+      <c r="E4" s="172" t="s">
         <v>442</v>
       </c>
-      <c r="F4" s="169"/>
-      <c r="G4" s="169"/>
-      <c r="H4" s="169"/>
-      <c r="I4" s="169"/>
-      <c r="J4" s="169"/>
-      <c r="K4" s="169"/>
-      <c r="L4" s="169"/>
-      <c r="M4" s="169"/>
-      <c r="N4" s="169"/>
-      <c r="O4" s="169"/>
-      <c r="P4" s="169"/>
-      <c r="Q4" s="169"/>
-      <c r="R4" s="169"/>
-      <c r="S4" s="169"/>
-      <c r="T4" s="169"/>
+      <c r="F4" s="172"/>
+      <c r="G4" s="172"/>
+      <c r="H4" s="172"/>
+      <c r="I4" s="172"/>
+      <c r="J4" s="172"/>
+      <c r="K4" s="172"/>
+      <c r="L4" s="172"/>
+      <c r="M4" s="172"/>
+      <c r="N4" s="172"/>
+      <c r="O4" s="172"/>
+      <c r="P4" s="172"/>
+      <c r="Q4" s="172"/>
+      <c r="R4" s="172"/>
+      <c r="S4" s="172"/>
+      <c r="T4" s="172"/>
     </row>
     <row r="5" spans="2:20">
-      <c r="B5" s="169"/>
-      <c r="C5" s="169"/>
-      <c r="D5" s="169"/>
+      <c r="B5" s="172"/>
+      <c r="C5" s="172"/>
+      <c r="D5" s="172"/>
       <c r="E5" s="44">
         <v>0</v>
       </c>
@@ -28032,9 +28044,9 @@
       </c>
     </row>
     <row r="6" spans="2:20" ht="103.5" customHeight="1">
-      <c r="B6" s="169"/>
-      <c r="C6" s="169"/>
-      <c r="D6" s="169"/>
+      <c r="B6" s="172"/>
+      <c r="C6" s="172"/>
+      <c r="D6" s="172"/>
       <c r="E6" s="63" t="s">
         <v>440</v>
       </c>
@@ -28085,7 +28097,7 @@
       </c>
     </row>
     <row r="7" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B7" s="166" t="s">
+      <c r="B7" s="169" t="s">
         <v>441</v>
       </c>
       <c r="C7" s="44">
@@ -28144,7 +28156,7 @@
       </c>
     </row>
     <row r="8" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B8" s="167"/>
+      <c r="B8" s="170"/>
       <c r="C8" s="44">
         <v>1</v>
       </c>
@@ -28201,7 +28213,7 @@
       </c>
     </row>
     <row r="9" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B9" s="167"/>
+      <c r="B9" s="170"/>
       <c r="C9" s="44">
         <v>2</v>
       </c>
@@ -28258,7 +28270,7 @@
       </c>
     </row>
     <row r="10" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B10" s="167"/>
+      <c r="B10" s="170"/>
       <c r="C10" s="44">
         <v>3</v>
       </c>
@@ -28315,7 +28327,7 @@
       </c>
     </row>
     <row r="11" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B11" s="167"/>
+      <c r="B11" s="170"/>
       <c r="C11" s="44">
         <v>4</v>
       </c>
@@ -28372,7 +28384,7 @@
       </c>
     </row>
     <row r="12" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B12" s="167"/>
+      <c r="B12" s="170"/>
       <c r="C12" s="44">
         <v>5</v>
       </c>
@@ -28429,7 +28441,7 @@
       </c>
     </row>
     <row r="13" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B13" s="167"/>
+      <c r="B13" s="170"/>
       <c r="C13" s="44">
         <v>6</v>
       </c>
@@ -28486,7 +28498,7 @@
       </c>
     </row>
     <row r="14" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B14" s="167"/>
+      <c r="B14" s="170"/>
       <c r="C14" s="44">
         <v>7</v>
       </c>
@@ -28543,7 +28555,7 @@
       </c>
     </row>
     <row r="15" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B15" s="167"/>
+      <c r="B15" s="170"/>
       <c r="C15" s="44">
         <v>8</v>
       </c>
@@ -28600,7 +28612,7 @@
       </c>
     </row>
     <row r="16" spans="2:20" ht="31.5" customHeight="1">
-      <c r="B16" s="167"/>
+      <c r="B16" s="170"/>
       <c r="C16" s="44">
         <v>9</v>
       </c>
@@ -28657,7 +28669,7 @@
       </c>
     </row>
     <row r="17" spans="2:22" ht="31.5" customHeight="1">
-      <c r="B17" s="167"/>
+      <c r="B17" s="170"/>
       <c r="C17" s="44">
         <v>10</v>
       </c>
@@ -28714,7 +28726,7 @@
       </c>
     </row>
     <row r="18" spans="2:22" ht="31.5" customHeight="1">
-      <c r="B18" s="167"/>
+      <c r="B18" s="170"/>
       <c r="C18" s="44">
         <v>11</v>
       </c>
@@ -28771,7 +28783,7 @@
       </c>
     </row>
     <row r="19" spans="2:22" ht="31.5" customHeight="1">
-      <c r="B19" s="167"/>
+      <c r="B19" s="170"/>
       <c r="C19" s="44">
         <v>12</v>
       </c>
@@ -28828,7 +28840,7 @@
       </c>
     </row>
     <row r="20" spans="2:22" ht="31.5" customHeight="1">
-      <c r="B20" s="167"/>
+      <c r="B20" s="170"/>
       <c r="C20" s="44">
         <v>13</v>
       </c>
@@ -28885,7 +28897,7 @@
       </c>
     </row>
     <row r="21" spans="2:22" ht="31.5" customHeight="1">
-      <c r="B21" s="167"/>
+      <c r="B21" s="170"/>
       <c r="C21" s="44">
         <v>14</v>
       </c>
@@ -28944,7 +28956,7 @@
       <c r="V21" s="39"/>
     </row>
     <row r="22" spans="2:22" ht="31.5" customHeight="1">
-      <c r="B22" s="168"/>
+      <c r="B22" s="171"/>
       <c r="C22" s="44">
         <v>15</v>
       </c>
@@ -31950,7 +31962,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F837E406-9569-443C-823E-A0F068C6235A}">
-  <dimension ref="B2:P40"/>
+  <dimension ref="B2:P44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="38" customWidth="1"/>
@@ -31973,34 +31985,34 @@
       </c>
     </row>
     <row r="3" spans="2:16">
-      <c r="B3" s="191" t="s">
+      <c r="B3" s="196" t="s">
         <v>489</v>
       </c>
-      <c r="C3" s="204" t="s">
+      <c r="C3" s="191" t="s">
         <v>488</v>
       </c>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="202"/>
-      <c r="G3" s="202"/>
-      <c r="H3" s="205"/>
-      <c r="I3" s="201" t="s">
+      <c r="D3" s="189"/>
+      <c r="E3" s="189"/>
+      <c r="F3" s="189"/>
+      <c r="G3" s="189"/>
+      <c r="H3" s="192"/>
+      <c r="I3" s="188" t="s">
         <v>487</v>
       </c>
-      <c r="J3" s="202"/>
-      <c r="K3" s="202"/>
-      <c r="L3" s="202"/>
-      <c r="M3" s="202"/>
-      <c r="N3" s="203"/>
+      <c r="J3" s="189"/>
+      <c r="K3" s="189"/>
+      <c r="L3" s="189"/>
+      <c r="M3" s="189"/>
+      <c r="N3" s="190"/>
       <c r="O3" s="104" t="s">
         <v>486</v>
       </c>
-      <c r="P3" s="197" t="s">
+      <c r="P3" s="185" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="4" spans="2:16" ht="15.75" thickBot="1">
-      <c r="B4" s="192"/>
+      <c r="B4" s="197"/>
       <c r="C4" s="105" t="s">
         <v>373</v>
       </c>
@@ -32040,7 +32052,7 @@
       <c r="O4" s="110" t="s">
         <v>479</v>
       </c>
-      <c r="P4" s="198"/>
+      <c r="P4" s="186"/>
     </row>
     <row r="5" spans="2:16" ht="15.75" thickTop="1">
       <c r="B5" s="64" t="s">
@@ -32116,12 +32128,12 @@
         <f t="shared" si="0"/>
         <v>0x01</v>
       </c>
-      <c r="J6" s="199" t="s">
+      <c r="J6" s="176" t="s">
         <v>508</v>
       </c>
-      <c r="K6" s="199"/>
-      <c r="L6" s="199"/>
-      <c r="M6" s="199"/>
+      <c r="K6" s="176"/>
+      <c r="L6" s="176"/>
+      <c r="M6" s="176"/>
       <c r="N6" s="77" t="s">
         <v>492</v>
       </c>
@@ -32158,12 +32170,12 @@
         <f t="shared" si="0"/>
         <v>0x02</v>
       </c>
-      <c r="J7" s="199" t="s">
+      <c r="J7" s="176" t="s">
         <v>523</v>
       </c>
-      <c r="K7" s="199"/>
-      <c r="L7" s="199"/>
-      <c r="M7" s="199"/>
+      <c r="K7" s="176"/>
+      <c r="L7" s="176"/>
+      <c r="M7" s="176"/>
       <c r="N7" s="77" t="s">
         <v>492</v>
       </c>
@@ -32200,12 +32212,12 @@
         <f t="shared" si="0"/>
         <v>0x03</v>
       </c>
-      <c r="J8" s="199" t="s">
+      <c r="J8" s="176" t="s">
         <v>506</v>
       </c>
-      <c r="K8" s="199"/>
-      <c r="L8" s="199"/>
-      <c r="M8" s="199"/>
+      <c r="K8" s="176"/>
+      <c r="L8" s="176"/>
+      <c r="M8" s="176"/>
       <c r="N8" s="77" t="s">
         <v>492</v>
       </c>
@@ -32242,14 +32254,14 @@
         <f t="shared" si="0"/>
         <v>0x04</v>
       </c>
-      <c r="J9" s="199" t="s">
+      <c r="J9" s="176" t="s">
         <v>503</v>
       </c>
-      <c r="K9" s="199"/>
-      <c r="L9" s="199" t="s">
+      <c r="K9" s="176"/>
+      <c r="L9" s="176" t="s">
         <v>502</v>
       </c>
-      <c r="M9" s="199"/>
+      <c r="M9" s="176"/>
       <c r="N9" s="77" t="s">
         <v>492</v>
       </c>
@@ -32411,12 +32423,12 @@
       <c r="C13" s="73" t="s">
         <v>564</v>
       </c>
-      <c r="D13" s="200" t="s">
+      <c r="D13" s="187" t="s">
         <v>508</v>
       </c>
-      <c r="E13" s="200"/>
-      <c r="F13" s="200"/>
-      <c r="G13" s="200"/>
+      <c r="E13" s="187"/>
+      <c r="F13" s="187"/>
+      <c r="G13" s="187"/>
       <c r="H13" s="103" t="s">
         <v>492</v>
       </c>
@@ -32501,12 +32513,12 @@
       <c r="C15" s="73" t="s">
         <v>566</v>
       </c>
-      <c r="D15" s="199" t="s">
+      <c r="D15" s="176" t="s">
         <v>506</v>
       </c>
-      <c r="E15" s="199"/>
-      <c r="F15" s="199"/>
-      <c r="G15" s="199"/>
+      <c r="E15" s="176"/>
+      <c r="F15" s="176"/>
+      <c r="G15" s="176"/>
       <c r="H15" s="75" t="s">
         <v>492</v>
       </c>
@@ -32543,14 +32555,14 @@
       <c r="C16" s="73" t="s">
         <v>567</v>
       </c>
-      <c r="D16" s="199" t="s">
+      <c r="D16" s="176" t="s">
         <v>503</v>
       </c>
-      <c r="E16" s="199"/>
-      <c r="F16" s="199" t="s">
+      <c r="E16" s="176"/>
+      <c r="F16" s="176" t="s">
         <v>502</v>
       </c>
-      <c r="G16" s="199"/>
+      <c r="G16" s="176"/>
       <c r="H16" s="75" t="s">
         <v>492</v>
       </c>
@@ -32732,34 +32744,34 @@
       <c r="D21" s="58"/>
     </row>
     <row r="22" spans="2:16">
-      <c r="B22" s="193" t="s">
+      <c r="B22" s="198" t="s">
         <v>489</v>
       </c>
-      <c r="C22" s="176" t="s">
+      <c r="C22" s="207" t="s">
         <v>488</v>
       </c>
-      <c r="D22" s="177"/>
-      <c r="E22" s="177"/>
-      <c r="F22" s="177"/>
-      <c r="G22" s="177"/>
-      <c r="H22" s="177"/>
-      <c r="I22" s="177"/>
-      <c r="J22" s="178"/>
-      <c r="K22" s="176" t="s">
+      <c r="D22" s="208"/>
+      <c r="E22" s="208"/>
+      <c r="F22" s="208"/>
+      <c r="G22" s="208"/>
+      <c r="H22" s="208"/>
+      <c r="I22" s="208"/>
+      <c r="J22" s="209"/>
+      <c r="K22" s="207" t="s">
         <v>487</v>
       </c>
-      <c r="L22" s="177"/>
-      <c r="M22" s="177"/>
-      <c r="N22" s="178"/>
+      <c r="L22" s="208"/>
+      <c r="M22" s="208"/>
+      <c r="N22" s="209"/>
       <c r="O22" s="104" t="s">
         <v>486</v>
       </c>
-      <c r="P22" s="206" t="s">
+      <c r="P22" s="173" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="23" spans="2:16" ht="15.75" thickBot="1">
-      <c r="B23" s="194"/>
+      <c r="B23" s="199"/>
       <c r="C23" s="111" t="s">
         <v>373</v>
       </c>
@@ -32775,21 +32787,21 @@
       <c r="G23" s="113" t="s">
         <v>482</v>
       </c>
-      <c r="H23" s="208" t="s">
+      <c r="H23" s="177" t="s">
         <v>481</v>
       </c>
-      <c r="I23" s="180"/>
-      <c r="J23" s="181"/>
-      <c r="K23" s="179" t="s">
+      <c r="I23" s="178"/>
+      <c r="J23" s="179"/>
+      <c r="K23" s="210" t="s">
         <v>480</v>
       </c>
-      <c r="L23" s="180"/>
-      <c r="M23" s="180"/>
-      <c r="N23" s="181"/>
+      <c r="L23" s="178"/>
+      <c r="M23" s="178"/>
+      <c r="N23" s="179"/>
       <c r="O23" s="110" t="s">
         <v>479</v>
       </c>
-      <c r="P23" s="207"/>
+      <c r="P23" s="174"/>
     </row>
     <row r="24" spans="2:16" ht="15.75" thickTop="1">
       <c r="B24" s="98" t="s">
@@ -32810,17 +32822,17 @@
       <c r="G24" s="57" t="s">
         <v>74</v>
       </c>
-      <c r="H24" s="209" t="s">
+      <c r="H24" s="180" t="s">
         <v>571</v>
       </c>
-      <c r="I24" s="185"/>
-      <c r="J24" s="186"/>
-      <c r="K24" s="184" t="s">
+      <c r="I24" s="181"/>
+      <c r="J24" s="182"/>
+      <c r="K24" s="212" t="s">
         <v>571</v>
       </c>
-      <c r="L24" s="185"/>
-      <c r="M24" s="185"/>
-      <c r="N24" s="186"/>
+      <c r="L24" s="181"/>
+      <c r="M24" s="181"/>
+      <c r="N24" s="182"/>
       <c r="O24" s="55" t="s">
         <v>477</v>
       </c>
@@ -32847,17 +32859,17 @@
       <c r="G25" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="H25" s="190" t="s">
+      <c r="H25" s="175" t="s">
         <v>571</v>
       </c>
-      <c r="I25" s="188"/>
-      <c r="J25" s="189"/>
-      <c r="K25" s="187" t="s">
+      <c r="I25" s="183"/>
+      <c r="J25" s="184"/>
+      <c r="K25" s="202" t="s">
         <v>571</v>
       </c>
-      <c r="L25" s="188"/>
-      <c r="M25" s="188"/>
-      <c r="N25" s="189"/>
+      <c r="L25" s="183"/>
+      <c r="M25" s="183"/>
+      <c r="N25" s="184"/>
       <c r="O25" s="52" t="s">
         <v>460</v>
       </c>
@@ -32884,17 +32896,17 @@
       <c r="G26" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="H26" s="190" t="s">
+      <c r="H26" s="175" t="s">
         <v>571</v>
       </c>
-      <c r="I26" s="188"/>
-      <c r="J26" s="189"/>
-      <c r="K26" s="187" t="s">
+      <c r="I26" s="183"/>
+      <c r="J26" s="184"/>
+      <c r="K26" s="202" t="s">
         <v>571</v>
       </c>
-      <c r="L26" s="188"/>
-      <c r="M26" s="188"/>
-      <c r="N26" s="189"/>
+      <c r="L26" s="183"/>
+      <c r="M26" s="183"/>
+      <c r="N26" s="184"/>
       <c r="O26" s="52" t="s">
         <v>460</v>
       </c>
@@ -32921,17 +32933,17 @@
       <c r="G27" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="H27" s="190" t="s">
+      <c r="H27" s="175" t="s">
         <v>571</v>
       </c>
-      <c r="I27" s="188"/>
-      <c r="J27" s="189"/>
-      <c r="K27" s="187" t="s">
+      <c r="I27" s="183"/>
+      <c r="J27" s="184"/>
+      <c r="K27" s="202" t="s">
         <v>571</v>
       </c>
-      <c r="L27" s="188"/>
-      <c r="M27" s="188"/>
-      <c r="N27" s="189"/>
+      <c r="L27" s="183"/>
+      <c r="M27" s="183"/>
+      <c r="N27" s="184"/>
       <c r="O27" s="52" t="s">
         <v>460</v>
       </c>
@@ -32958,17 +32970,17 @@
       <c r="G28" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="H28" s="190" t="s">
+      <c r="H28" s="175" t="s">
         <v>571</v>
       </c>
-      <c r="I28" s="188"/>
-      <c r="J28" s="189"/>
-      <c r="K28" s="187" t="s">
+      <c r="I28" s="183"/>
+      <c r="J28" s="184"/>
+      <c r="K28" s="202" t="s">
         <v>571</v>
       </c>
-      <c r="L28" s="188"/>
-      <c r="M28" s="188"/>
-      <c r="N28" s="189"/>
+      <c r="L28" s="183"/>
+      <c r="M28" s="183"/>
+      <c r="N28" s="184"/>
       <c r="O28" s="52" t="s">
         <v>460</v>
       </c>
@@ -32983,23 +32995,23 @@
       <c r="C29" s="61" t="s">
         <v>554</v>
       </c>
-      <c r="D29" s="169" t="s">
+      <c r="D29" s="172" t="s">
         <v>465</v>
       </c>
-      <c r="E29" s="169"/>
-      <c r="F29" s="169"/>
-      <c r="G29" s="190"/>
-      <c r="H29" s="190" t="s">
+      <c r="E29" s="172"/>
+      <c r="F29" s="172"/>
+      <c r="G29" s="175"/>
+      <c r="H29" s="175" t="s">
         <v>571</v>
       </c>
-      <c r="I29" s="188"/>
-      <c r="J29" s="189"/>
-      <c r="K29" s="187" t="s">
+      <c r="I29" s="183"/>
+      <c r="J29" s="184"/>
+      <c r="K29" s="202" t="s">
         <v>571</v>
       </c>
-      <c r="L29" s="188"/>
-      <c r="M29" s="188"/>
-      <c r="N29" s="189"/>
+      <c r="L29" s="183"/>
+      <c r="M29" s="183"/>
+      <c r="N29" s="184"/>
       <c r="O29" s="52" t="s">
         <v>460</v>
       </c>
@@ -33014,23 +33026,23 @@
       <c r="C30" s="61" t="s">
         <v>555</v>
       </c>
-      <c r="D30" s="169" t="s">
-        <v>465</v>
-      </c>
-      <c r="E30" s="169"/>
-      <c r="F30" s="169"/>
-      <c r="G30" s="190"/>
-      <c r="H30" s="190" t="s">
+      <c r="D30" s="172" t="s">
+        <v>750</v>
+      </c>
+      <c r="E30" s="172"/>
+      <c r="F30" s="172"/>
+      <c r="G30" s="175"/>
+      <c r="H30" s="175" t="s">
         <v>455</v>
       </c>
-      <c r="I30" s="188"/>
-      <c r="J30" s="189"/>
-      <c r="K30" s="187" t="s">
+      <c r="I30" s="183"/>
+      <c r="J30" s="184"/>
+      <c r="K30" s="202" t="s">
         <v>455</v>
       </c>
-      <c r="L30" s="188"/>
-      <c r="M30" s="188"/>
-      <c r="N30" s="189"/>
+      <c r="L30" s="183"/>
+      <c r="M30" s="183"/>
+      <c r="N30" s="184"/>
       <c r="O30" s="52" t="s">
         <v>460</v>
       </c>
@@ -33045,23 +33057,23 @@
       <c r="C31" s="61" t="s">
         <v>556</v>
       </c>
-      <c r="D31" s="169" t="s">
-        <v>465</v>
-      </c>
-      <c r="E31" s="169"/>
-      <c r="F31" s="169"/>
-      <c r="G31" s="190"/>
-      <c r="H31" s="190" t="s">
+      <c r="D31" s="172" t="s">
+        <v>750</v>
+      </c>
+      <c r="E31" s="172"/>
+      <c r="F31" s="172"/>
+      <c r="G31" s="175"/>
+      <c r="H31" s="175" t="s">
         <v>455</v>
       </c>
-      <c r="I31" s="188"/>
-      <c r="J31" s="189"/>
-      <c r="K31" s="187" t="s">
+      <c r="I31" s="183"/>
+      <c r="J31" s="184"/>
+      <c r="K31" s="202" t="s">
         <v>455</v>
       </c>
-      <c r="L31" s="188"/>
-      <c r="M31" s="188"/>
-      <c r="N31" s="189"/>
+      <c r="L31" s="183"/>
+      <c r="M31" s="183"/>
+      <c r="N31" s="184"/>
       <c r="O31" s="52" t="s">
         <v>460</v>
       </c>
@@ -33076,23 +33088,23 @@
       <c r="C32" s="60" t="s">
         <v>557</v>
       </c>
-      <c r="D32" s="195" t="s">
+      <c r="D32" s="200" t="s">
         <v>465</v>
       </c>
-      <c r="E32" s="195"/>
-      <c r="F32" s="195"/>
-      <c r="G32" s="196"/>
-      <c r="H32" s="182" t="s">
+      <c r="E32" s="200"/>
+      <c r="F32" s="200"/>
+      <c r="G32" s="201"/>
+      <c r="H32" s="193" t="s">
         <v>455</v>
       </c>
-      <c r="I32" s="171"/>
-      <c r="J32" s="172"/>
-      <c r="K32" s="170" t="s">
+      <c r="I32" s="194"/>
+      <c r="J32" s="195"/>
+      <c r="K32" s="203" t="s">
         <v>455</v>
       </c>
-      <c r="L32" s="171"/>
-      <c r="M32" s="171"/>
-      <c r="N32" s="172"/>
+      <c r="L32" s="194"/>
+      <c r="M32" s="194"/>
+      <c r="N32" s="195"/>
       <c r="O32" s="100" t="s">
         <v>446</v>
       </c>
@@ -33107,23 +33119,23 @@
       <c r="C33" s="60" t="s">
         <v>558</v>
       </c>
-      <c r="D33" s="195" t="s">
+      <c r="D33" s="200" t="s">
         <v>465</v>
       </c>
-      <c r="E33" s="195"/>
-      <c r="F33" s="195"/>
-      <c r="G33" s="196"/>
-      <c r="H33" s="182" t="s">
+      <c r="E33" s="200"/>
+      <c r="F33" s="200"/>
+      <c r="G33" s="201"/>
+      <c r="H33" s="193" t="s">
         <v>455</v>
       </c>
-      <c r="I33" s="171"/>
-      <c r="J33" s="172"/>
-      <c r="K33" s="170" t="s">
+      <c r="I33" s="194"/>
+      <c r="J33" s="195"/>
+      <c r="K33" s="203" t="s">
         <v>455</v>
       </c>
-      <c r="L33" s="171"/>
-      <c r="M33" s="171"/>
-      <c r="N33" s="172"/>
+      <c r="L33" s="194"/>
+      <c r="M33" s="194"/>
+      <c r="N33" s="195"/>
       <c r="O33" s="100" t="s">
         <v>446</v>
       </c>
@@ -33150,17 +33162,17 @@
       <c r="G34" s="49" t="s">
         <v>74</v>
       </c>
-      <c r="H34" s="182" t="s">
+      <c r="H34" s="193" t="s">
         <v>571</v>
       </c>
-      <c r="I34" s="171"/>
-      <c r="J34" s="172"/>
-      <c r="K34" s="170" t="s">
+      <c r="I34" s="194"/>
+      <c r="J34" s="195"/>
+      <c r="K34" s="203" t="s">
         <v>571</v>
       </c>
-      <c r="L34" s="171"/>
-      <c r="M34" s="171"/>
-      <c r="N34" s="172"/>
+      <c r="L34" s="194"/>
+      <c r="M34" s="194"/>
+      <c r="N34" s="195"/>
       <c r="O34" s="100" t="s">
         <v>446</v>
       </c>
@@ -33187,17 +33199,17 @@
       <c r="G35" s="49" t="s">
         <v>74</v>
       </c>
-      <c r="H35" s="182" t="s">
+      <c r="H35" s="193" t="s">
         <v>571</v>
       </c>
-      <c r="I35" s="171"/>
-      <c r="J35" s="172"/>
-      <c r="K35" s="170" t="s">
+      <c r="I35" s="194"/>
+      <c r="J35" s="195"/>
+      <c r="K35" s="203" t="s">
         <v>571</v>
       </c>
-      <c r="L35" s="171"/>
-      <c r="M35" s="171"/>
-      <c r="N35" s="172"/>
+      <c r="L35" s="194"/>
+      <c r="M35" s="194"/>
+      <c r="N35" s="195"/>
       <c r="O35" s="100" t="s">
         <v>446</v>
       </c>
@@ -33224,17 +33236,17 @@
       <c r="G36" s="49" t="s">
         <v>74</v>
       </c>
-      <c r="H36" s="182" t="s">
+      <c r="H36" s="193" t="s">
         <v>571</v>
       </c>
-      <c r="I36" s="171"/>
-      <c r="J36" s="172"/>
-      <c r="K36" s="170" t="s">
+      <c r="I36" s="194"/>
+      <c r="J36" s="195"/>
+      <c r="K36" s="203" t="s">
         <v>571</v>
       </c>
-      <c r="L36" s="171"/>
-      <c r="M36" s="171"/>
-      <c r="N36" s="172"/>
+      <c r="L36" s="194"/>
+      <c r="M36" s="194"/>
+      <c r="N36" s="195"/>
       <c r="O36" s="100" t="s">
         <v>446</v>
       </c>
@@ -33261,17 +33273,17 @@
       <c r="G37" s="46" t="s">
         <v>74</v>
       </c>
-      <c r="H37" s="183" t="s">
+      <c r="H37" s="211" t="s">
         <v>571</v>
       </c>
-      <c r="I37" s="174"/>
-      <c r="J37" s="175"/>
-      <c r="K37" s="173" t="s">
+      <c r="I37" s="205"/>
+      <c r="J37" s="206"/>
+      <c r="K37" s="204" t="s">
         <v>571</v>
       </c>
-      <c r="L37" s="174"/>
-      <c r="M37" s="174"/>
-      <c r="N37" s="175"/>
+      <c r="L37" s="205"/>
+      <c r="M37" s="205"/>
+      <c r="N37" s="206"/>
       <c r="O37" s="101" t="s">
         <v>446</v>
       </c>
@@ -33289,44 +33301,23 @@
         <v>443</v>
       </c>
     </row>
+    <row r="42" spans="2:16">
+      <c r="K42" s="38" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="43" spans="2:16">
+      <c r="K43" s="38" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="44" spans="2:16">
+      <c r="K44" s="38" t="s">
+        <v>753</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="P22:P23"/>
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="D15:G15"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D13:G13"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="I3:N3"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="H30:J30"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="H32:J32"/>
-    <mergeCell ref="H33:J33"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="D33:G33"/>
-    <mergeCell ref="D32:G32"/>
-    <mergeCell ref="D31:G31"/>
-    <mergeCell ref="D30:G30"/>
-    <mergeCell ref="K31:N31"/>
-    <mergeCell ref="K32:N32"/>
-    <mergeCell ref="K33:N33"/>
-    <mergeCell ref="K34:N34"/>
-    <mergeCell ref="K35:N35"/>
     <mergeCell ref="K36:N36"/>
     <mergeCell ref="K37:N37"/>
     <mergeCell ref="C22:J22"/>
@@ -33343,6 +33334,42 @@
     <mergeCell ref="K28:N28"/>
     <mergeCell ref="K29:N29"/>
     <mergeCell ref="K30:N30"/>
+    <mergeCell ref="K31:N31"/>
+    <mergeCell ref="K32:N32"/>
+    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="K34:N34"/>
+    <mergeCell ref="K35:N35"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="H32:J32"/>
+    <mergeCell ref="H33:J33"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="D33:G33"/>
+    <mergeCell ref="D32:G32"/>
+    <mergeCell ref="D31:G31"/>
+    <mergeCell ref="D30:G30"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="I3:N3"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="P22:P23"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="H25:J25"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="H29:J29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -33366,44 +33393,44 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10">
-      <c r="B2" s="213" t="s">
+      <c r="B2" s="216" t="s">
         <v>616</v>
       </c>
-      <c r="C2" s="212" t="s">
+      <c r="C2" s="215" t="s">
         <v>615</v>
       </c>
-      <c r="D2" s="213" t="s">
+      <c r="D2" s="216" t="s">
         <v>373</v>
       </c>
-      <c r="E2" s="212" t="s">
+      <c r="E2" s="215" t="s">
         <v>608</v>
       </c>
-      <c r="F2" s="210"/>
-      <c r="G2" s="210" t="s">
+      <c r="F2" s="213"/>
+      <c r="G2" s="213" t="s">
         <v>631</v>
       </c>
-      <c r="H2" s="210" t="s">
+      <c r="H2" s="213" t="s">
         <v>730</v>
       </c>
       <c r="I2" s="114" t="s">
         <v>486</v>
       </c>
-      <c r="J2" s="212" t="s">
+      <c r="J2" s="215" t="s">
         <v>609</v>
       </c>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="213"/>
-      <c r="C3" s="212"/>
-      <c r="D3" s="213"/>
-      <c r="E3" s="212"/>
-      <c r="F3" s="211"/>
-      <c r="G3" s="211"/>
-      <c r="H3" s="211"/>
+      <c r="B3" s="216"/>
+      <c r="C3" s="215"/>
+      <c r="D3" s="216"/>
+      <c r="E3" s="215"/>
+      <c r="F3" s="214"/>
+      <c r="G3" s="214"/>
+      <c r="H3" s="214"/>
       <c r="I3" s="115" t="s">
         <v>479</v>
       </c>
-      <c r="J3" s="212"/>
+      <c r="J3" s="215"/>
     </row>
     <row r="4" spans="2:10">
       <c r="B4" s="128" t="s">
@@ -34377,62 +34404,62 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="6" spans="3:3">
-      <c r="C6" s="214" t="s">
+      <c r="C6" s="164" t="s">
         <v>739</v>
       </c>
     </row>
     <row r="7" spans="3:3">
-      <c r="C7" s="215" t="s">
+      <c r="C7" s="165" t="s">
         <v>740</v>
       </c>
     </row>
     <row r="8" spans="3:3">
-      <c r="C8" s="215" t="s">
+      <c r="C8" s="165" t="s">
         <v>741</v>
       </c>
     </row>
     <row r="9" spans="3:3">
-      <c r="C9" s="216" t="s">
+      <c r="C9" s="166" t="s">
         <v>742</v>
       </c>
     </row>
     <row r="10" spans="3:3">
-      <c r="C10" s="216" t="s">
+      <c r="C10" s="166" t="s">
         <v>743</v>
       </c>
     </row>
     <row r="11" spans="3:3">
-      <c r="C11" s="216" t="s">
+      <c r="C11" s="166" t="s">
         <v>743</v>
       </c>
     </row>
     <row r="12" spans="3:3">
-      <c r="C12" s="216" t="s">
+      <c r="C12" s="166" t="s">
         <v>744</v>
       </c>
     </row>
     <row r="13" spans="3:3">
-      <c r="C13" s="216" t="s">
+      <c r="C13" s="166" t="s">
         <v>745</v>
       </c>
     </row>
     <row r="14" spans="3:3">
-      <c r="C14" s="216" t="s">
+      <c r="C14" s="166" t="s">
         <v>746</v>
       </c>
     </row>
     <row r="15" spans="3:3">
-      <c r="C15" s="216" t="s">
+      <c r="C15" s="166" t="s">
         <v>747</v>
       </c>
     </row>
     <row r="17" spans="3:3">
-      <c r="C17" s="214" t="s">
+      <c r="C17" s="164" t="s">
         <v>748</v>
       </c>
     </row>
     <row r="18" spans="3:3">
-      <c r="C18" s="215" t="s">
+      <c r="C18" s="165" t="s">
         <v>749</v>
       </c>
     </row>
@@ -35114,46 +35141,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="13" customFormat="1" ht="12" customHeight="1">
-      <c r="A1" s="164" t="s">
+      <c r="A1" s="167" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="164"/>
-      <c r="C1" s="164"/>
-      <c r="D1" s="164"/>
-      <c r="E1" s="164"/>
-      <c r="F1" s="164"/>
+      <c r="B1" s="167"/>
+      <c r="C1" s="167"/>
+      <c r="D1" s="167"/>
+      <c r="E1" s="167"/>
+      <c r="F1" s="167"/>
     </row>
     <row r="2" spans="1:22" s="13" customFormat="1" ht="12" customHeight="1">
-      <c r="A2" s="164"/>
-      <c r="B2" s="164"/>
-      <c r="C2" s="164"/>
-      <c r="D2" s="164"/>
-      <c r="E2" s="164"/>
-      <c r="F2" s="164"/>
+      <c r="A2" s="167"/>
+      <c r="B2" s="167"/>
+      <c r="C2" s="167"/>
+      <c r="D2" s="167"/>
+      <c r="E2" s="167"/>
+      <c r="F2" s="167"/>
     </row>
     <row r="3" spans="1:22" s="13" customFormat="1" ht="12" customHeight="1">
-      <c r="A3" s="164"/>
-      <c r="B3" s="164"/>
-      <c r="C3" s="164"/>
-      <c r="D3" s="164"/>
-      <c r="E3" s="164"/>
-      <c r="F3" s="164"/>
+      <c r="A3" s="167"/>
+      <c r="B3" s="167"/>
+      <c r="C3" s="167"/>
+      <c r="D3" s="167"/>
+      <c r="E3" s="167"/>
+      <c r="F3" s="167"/>
     </row>
     <row r="4" spans="1:22" s="13" customFormat="1" ht="12" customHeight="1">
-      <c r="A4" s="164"/>
-      <c r="B4" s="164"/>
-      <c r="C4" s="164"/>
-      <c r="D4" s="164"/>
-      <c r="E4" s="164"/>
-      <c r="F4" s="164"/>
+      <c r="A4" s="167"/>
+      <c r="B4" s="167"/>
+      <c r="C4" s="167"/>
+      <c r="D4" s="167"/>
+      <c r="E4" s="167"/>
+      <c r="F4" s="167"/>
     </row>
     <row r="5" spans="1:22" s="13" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A5" s="164"/>
-      <c r="B5" s="164"/>
-      <c r="C5" s="164"/>
-      <c r="D5" s="164"/>
-      <c r="E5" s="164"/>
-      <c r="F5" s="164"/>
+      <c r="A5" s="167"/>
+      <c r="B5" s="167"/>
+      <c r="C5" s="167"/>
+      <c r="D5" s="167"/>
+      <c r="E5" s="167"/>
+      <c r="F5" s="167"/>
     </row>
     <row r="6" spans="1:22" ht="28.5" customHeight="1">
       <c r="A6" s="143" t="s">

</xml_diff>